<commit_message>
scrub sample workbook metadata
</commit_message>
<xml_diff>
--- a/tools/bulk_ping_monitor/devices.xlsx
+++ b/tools/bulk_ping_monitor/devices.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Azizul\Project 2026\Python Automation Tools\Network Engineer Offline Toolkit\Bulk Network Ping Monitor\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E165993C-B5CA-464D-B106-80D8A6716DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E471BEBE-3F5D-4403-AE6B-1EB50E4D6674}"/>

</xml_diff>